<commit_message>
feat(F-NAR-019): ATOM-DIF.BES.001-02 La boule de pâte d'Amir
</commit_message>
<xml_diff>
--- a/stories/arbres/ATOM-DIF.BES.001-02.xlsx
+++ b/stories/arbres/ATOM-DIF.BES.001-02.xlsx
@@ -544,7 +544,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>L'escargot de pâte d'Amir</t>
+          <t>La boule de pâte d'Amir</t>
         </is>
       </c>
     </row>
@@ -676,7 +676,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>atelier de pâte, puis nappe à la maison</t>
+          <t>atelier de pâte à l'école, table près de la fenêtre, cuisine à la maison</t>
         </is>
       </c>
     </row>
@@ -688,7 +688,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Amir, Victorina, papa, maman</t>
+          <t>Amir, papa, maman</t>
         </is>
       </c>
     </row>
@@ -846,7 +846,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Amir veut un escargot de pâte, tout en spirale. Victorina regarde d'abord. Le soir, un oiseau de cartes. Même calme, autre table.</t>
+          <t>Le robinet de l'atelier fait tic. Une goutte ronde tombe. Sur une petite boule, un éclat de boule brille. Amir veut sa boule ronde, maintenant, près de la vitre. Il serre trop fort : la pâte s'écrase, l'éclat saute. Il refuse de foncer, regarde, roule le même geste. Merci vécu. À la maison, une boule file vers la vitre. L'éclat de boule tient.</t>
         </is>
       </c>
     </row>
@@ -1189,17 +1189,17 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>La cour sent l'herbe coupée. Un arrosoir goutte sous le robinet. Dans l'atelier, la table est froide. Un rouleau de bois attend, tout lisse. Un morceau de pâte a déjà une oreille. Tu as vu l'oreille, Amir ? Elle sèche. Près de la fenêtre. Oui. On en fait un autre. Je veux un escargot. Tout en spirale. Une boule, puis on roule. En ce moment, Amir arrive à la table. La pâte est froide sous les doigts. Elle sent un peu la farine. Elle est molle. Oui. Froide et molle. Victorina reste près de la table. Elle regarde les mains, sans bouger. Ses doigts restent sur le bord. Elle ne prend pas encore de pâte. Victorina. Tu viens ? Victorina ne vient pas encore. Elle a besoin de calme. Tu peux dire la règle. L'arrosoir goutte encore, dehors. La spirale n'est pas commencée.</t>
+          <t>Le robinet de l'atelier fait tic. Une goutte tombe dans l'évier. Elle est ronde, presque. Dehors, la cour sent la terre mouillée. La vitre a des traces de pluie. Amir pose les mains sur la table. L'atelier sent le bois mouillé. Tu as vu la cour, par la vitre ? Elle est mouillée. Ça sent la terre. On reste un moment, ici. La table est froide, un peu collante. Un tas de pâte attend au milieu. Au bord, une poudre blanche dort. Une planche de bois attend sous la vitre. Une petite boule repose près du tas. Sur la boule, un éclat de boule brille. Il est blanc, maman. Tu le vois sur la pâte ? Oui, il brille. C'est une boule de pâte. Je veux la mienne, maintenant ! Tes mains, Amir. On les passe sous l'eau. L'eau est froide. Comme la pâte. Je veux une boule ronde. Tu la veux ronde ? Ronde comme la goutte. Près de la fenêtre, elle peut sécher. Oui, près de la vitre. En ce moment, Amir prend la pâte. Il en arrache un gros morceau. Ses paumes ferment trop fort. La pâte s'écrase entre les doigts. Elle devient plate, avec une fente. Ça ne veut pas. L'éclat de boule saute près de la poudre. Le sourire d'Amir disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Ses épaules tombent un peu. Papa s'accroupit à la même hauteur. Tu veux la boule ronde ? Oui, papa. Tes mains sont collantes ? Oui, maman. Tu tiens ma manche ? Oui. Amir veut recommencer tout de suite. Ses doigts foncent vers le tas. La pâte plate reste là, fendue. Je la veux maintenant !</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>La cour sent l'herbe coupée. Un arrosoir goutte sous le robinet. Dans l'atelier, la table est froide. Un rouleau de bois attend, tout lisse. Un morceau de pâte a déjà une oreille. Tu as vu l'oreille, Amir ? Elle sèche. Près de la fenêtre. Oui. On en fait un autre. Je veux un escargot. Tout en spirale. Une boule, puis on roule. En ce moment, Amir arrive à la table. La pâte est froide sous les doigts. Elle sent un peu la farine. Elle est molle. Oui. Froide et molle. Victorina reste près de la table. Elle regarde les mains, sans bouger. Ses doigts restent sur le bord. Elle ne prend pas encore de pâte. Victorina. Tu viens ? Victorina ne vient pas encore. Elle a besoin de calme. Tu peux dire la règle. L'arrosoir goutte encore, dehors. La spirale n'est pas commencée.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le robinet de l'atelier fait tic. Une goutte tombe dans l'évier. Elle est ronde, presque. Dehors, la cour sent la terre mouillée. La vitre a des traces de pluie. Amir pose les mains sur la table. L'atelier sent le bois mouillé. Tu as vu la cour, par la vitre ? Elle est mouillée. Ça sent la terre. On reste un moment, ici. La table est froide, un peu collante. Un tas de pâte attend au milieu. Au bord, une poudre blanche dort. Une planche de bois attend sous la vitre. Une petite boule repose près du tas. Sur la boule, un &lt;emphasis level="moderate"&gt;éclat de boule&lt;/emphasis&gt; brille. Il est blanc, maman. Tu le vois sur la pâte ? Oui, il brille. C'est une boule de pâte. Je veux la mienne, maintenant ! Tes mains, Amir. On les passe sous l'eau. L'eau est froide. Comme la pâte. Je veux une boule ronde. Tu la veux ronde ? Ronde comme la goutte. Près de la fenêtre, elle peut sécher. Oui, près de la vitre. En ce moment, Amir prend la pâte. Il en arrache un gros morceau. Ses paumes ferment trop fort. La pâte s'écrase entre les doigts. Elle devient plate, avec une fente. Ça ne veut pas. L'éclat de boule saute près de la poudre. Le sourire d'Amir disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Ses épaules tombent un peu. Papa s'accroupit à la même hauteur. Tu veux la boule ronde ? Oui, papa. Tes mains sont collantes ? Oui, maman. Tu tiens ma manche ? Oui. Amir veut recommencer tout de suite. Ses doigts foncent vers le tas. La pâte plate reste là, fendue. Je la veux maintenant !&lt;/prosody&gt;&lt;break time="500ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>Léo est à l'atelier pâte, à l'école. Maman est encore à la porte. La maîtresse explique. On roule une boule. On aplatit. Amina reste près de la table. Elle a besoin de calme. Léo va vers elle. Il va &lt;emphasis&gt;répéter&lt;/emphasis&gt; la règle. Léo dit : une boule, puis on aplatit. Amina écoute. Elle va observer d'abord. Elle regarde les mains. Elle ne joue pas encore. C'est possible. Plus tard, à la maison, papa sort un jeu de cartes. Amina s'assoit au bord. Léo se souvient. Il va répéter. Léo dit : on pioche, on montre, on pose. Amina observe d'abord. Puis elle pioche une carte. Maman dit : tu as su répéter. Observer d'abord, c'est possible. Même leçon, autre lieu. [pause]</t>
+          <t>Le robinet de l'atelier fait tic. Une goutte tombe dans l'évier. Elle est ronde, presque. Dehors, la cour sent la terre mouillée. La vitre a des traces de pluie. Amir pose les mains sur la table. L'atelier sent le bois mouillé. Tu as vu la cour, par la vitre ? Elle est mouillée. Ça sent la terre. On reste un moment, ici. La table est froide, un peu collante. Un tas de pâte attend au milieu. Au bord, une poudre blanche dort. Une planche de bois attend sous la vitre. Une petite boule repose près du tas. Sur la boule, un &lt;emphasis&gt;éclat de boule&lt;/emphasis&gt; brille. Il est blanc, maman. Tu le vois sur la pâte ? Oui, il brille. C'est une boule de pâte. Je veux la mienne, maintenant ! Tes mains, Amir. On les passe sous l'eau. L'eau est froide. Comme la pâte. Je veux une boule ronde. Tu la veux ronde ? Ronde comme la goutte. Près de la fenêtre, elle peut sécher. Oui, près de la vitre. En ce moment, Amir prend la pâte. Il en arrache un gros morceau. Ses paumes ferment trop fort. La pâte s'écrase entre les doigts. Elle devient plate, avec une fente. Ça ne veut pas. L'éclat de boule saute près de la poudre. Le sourire d'Amir disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Ses épaules tombent un peu. Papa s'accroupit à la même hauteur. Tu veux la boule ronde ? Oui, papa. Tes mains sont collantes ? Oui, maman. Tu tiens ma manche ? Oui. Amir veut recommencer tout de suite. Ses doigts foncent vers le tas. La pâte plate reste là, fendue. Je la veux maintenant ! [pause]</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr"/>
@@ -1246,7 +1246,7 @@
         </is>
       </c>
       <c r="Y2" s="2" t="n">
-        <v>148</v>
+        <v>142</v>
       </c>
       <c r="Z2" s="2" t="inlineStr">
         <is>
@@ -1254,10 +1254,10 @@
         </is>
       </c>
       <c r="AA2" s="2" t="n">
-        <v>0.96</v>
+        <v>0.98</v>
       </c>
       <c r="AB2" s="2" t="n">
-        <v>1.22</v>
+        <v>1.12</v>
       </c>
       <c r="AC2" s="2" t="inlineStr">
         <is>
@@ -1280,30 +1280,30 @@
       </c>
       <c r="AH2" s="2" t="inlineStr">
         <is>
-          <t>répéter</t>
+          <t>éclat de boule</t>
         </is>
       </c>
       <c r="AI2" s="2" t="n">
         <v>0</v>
       </c>
       <c r="AJ2" s="2" t="n">
-        <v>400</v>
+        <v>500</v>
       </c>
       <c r="AK2" s="2" t="n">
-        <v>280</v>
+        <v>260</v>
       </c>
       <c r="AL2" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>warm</t>
         </is>
       </c>
       <c r="AM2" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>storytelling</t>
         </is>
       </c>
       <c r="AN2" s="2" t="n">
-        <v>0.333</v>
+        <v>0.36</v>
       </c>
       <c r="AO2" s="2" t="inlineStr"/>
       <c r="AP2" s="2" t="inlineStr">
@@ -1312,10 +1312,10 @@
         </is>
       </c>
       <c r="AQ2" s="2" t="n">
-        <v>0.96</v>
+        <v>0.98</v>
       </c>
       <c r="AR2" s="2" t="n">
-        <v>0.96</v>
+        <v>0.98</v>
       </c>
       <c r="AS2" s="2" t="n">
         <v>100</v>
@@ -1326,44 +1326,70 @@
       <c r="AU2" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="AV2" s="2" t="inlineStr"/>
+      <c r="AV2" s="2" t="inlineStr">
+        <is>
+          <t>arc=installation; intention=émerveiller puis tendre; emotion=impatience puis découragement; intensite=2; destinataire=enfant; sous_texte=il_veut_sa_boule_ronde_maintenant; tempo=naturel puis resserré; sourire=léger puis aucun; respiration=ample puis retenue</t>
+        </is>
+      </c>
       <c r="AW2" t="inlineStr">
         <is>
-          <t>narrateur|La cour sent l'herbe coupée.
-narrateur|Un arrosoir goutte sous le robinet.
-narrateur|Dans l'atelier, la table est froide.
-narrateur|Un rouleau de bois attend, tout lisse.
-narrateur|Un morceau de pâte a déjà une oreille.
-maman|Tu as vu l'oreille, Amir ?
-enfant-m|Elle sèche.
-enfant-m|Près de la fenêtre.
-maman|Oui.
-maman|On en fait un autre.
-enfant-m|Je veux un escargot.
-enfant-m|Tout en spirale.
-maman|Une boule, puis on roule.
-narrateur|En ce moment, Amir arrive à la table.
-narrateur|La pâte est froide sous les doigts.
-narrateur|Elle sent un peu la farine.
-enfant-m|Elle est molle.
-maman|Oui.
-maman|Froide et molle.
-narrateur|Victorina reste près de la table.
-narrateur|Elle regarde les mains, sans bouger.
-narrateur|Ses doigts restent sur le bord.
-narrateur|Elle ne prend pas encore de pâte.
-enfant-m|Victorina.
-enfant-m|Tu viens ?
-narrateur|Victorina ne vient pas encore.
-maman|Elle a besoin de calme.
-maman|Tu peux dire la règle.
-narrateur|L'arrosoir goutte encore, dehors.
-narrateur|La spirale n'est pas commencée.</t>
+          <t>narrateur|Le robinet de l'atelier fait tic.
+narrateur|Une goutte tombe dans l'évier.
+narrateur|Elle est ronde, presque.
+narrateur|Dehors, la cour sent la terre mouillée.
+narrateur|La vitre a des traces de pluie.
+narrateur|Amir pose les mains sur la table.
+narrateur|L'atelier sent le bois mouillé.
+maman|Tu as vu la cour, par la vitre ?
+enfant-m|Elle est mouillée.
+enfant-m|Ça sent la terre.
+papa|On reste un moment, ici.
+narrateur|La table est froide, un peu collante.
+narrateur|Un tas de pâte attend au milieu.
+narrateur|Au bord, une poudre blanche dort.
+narrateur|Une planche de bois attend sous la vitre.
+narrateur|Une petite boule repose près du tas.
+narrateur|Sur la boule, un éclat de boule brille.
+enfant-m|Il est blanc, maman.
+maman|Tu le vois sur la pâte ?
+enfant-m|Oui, il brille.
+papa|C'est une boule de pâte.
+enfant-m|Je veux la mienne, maintenant !
+maman|Tes mains, Amir.
+maman|On les passe sous l'eau.
+enfant-m|L'eau est froide.
+papa|Comme la pâte.
+enfant-m|Je veux une boule ronde.
+maman|Tu la veux ronde ?
+enfant-m|Ronde comme la goutte.
+papa|Près de la fenêtre, elle peut sécher.
+enfant-m|Oui, près de la vitre.
+narrateur|En ce moment, Amir prend la pâte.
+narrateur|Il en arrache un gros morceau.
+narrateur|Ses paumes ferment trop fort.
+narrateur|La pâte s'écrase entre les doigts.
+narrateur|Elle devient plate, avec une fente.
+enfant-m|Ça ne veut pas.
+narrateur|L'éclat de boule saute près de la poudre.
+narrateur|Le sourire d'Amir disparaît.
+narrateur|Dans sa poitrine, l'envie et l'inquiétude se bousculent.
+narrateur|Ses épaules tombent un peu.
+narrateur|Papa s'accroupit à la même hauteur.
+papa|Tu veux la boule ronde ?
+enfant-m|Oui, papa.
+maman|Tes mains sont collantes ?
+enfant-m|Oui, maman.
+papa|Tu tiens ma manche ?
+enfant-m|Oui.
+narrateur|Amir veut recommencer tout de suite.
+narrateur|Ses doigts foncent vers le tas.
+narrateur|La pâte plate reste là, fendue.
+enfant-m|Je la veux maintenant !</t>
         </is>
       </c>
       <c r="AX2" t="inlineStr">
         <is>
-          <t>pate,robinet</t>
+          <t>pate,robinet,goutte</t>
         </is>
       </c>
     </row>
@@ -1390,17 +1416,17 @@
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>Victorina a besoin de calme. Que peut-on faire ?</t>
+          <t>Amir a besoin de calme. Que peut-on faire ?</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Victorina a besoin de calme. Que peut-on faire ?</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;Amir a besoin de &lt;emphasis level="moderate"&gt;calme&lt;/emphasis&gt;. Que peut-on faire ?&lt;/prosody&gt;&lt;break time="700ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>Amina a besoin de calme. Que peut-on faire ?</t>
+          <t>&lt;soft&gt;&lt;slow&gt;Amir a besoin de &lt;emphasis&gt;calme&lt;/emphasis&gt;. Que peut-on faire ?&lt;/slow&gt;&lt;/soft&gt; [pause]</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -1425,7 +1451,7 @@
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>On peut répéter. On peut observer d'abord. Que fait-on ?</t>
+          <t>On peut répéter. On peut observer d'abord. Que fait Amir ?</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr"/>
@@ -1463,18 +1489,18 @@
         </is>
       </c>
       <c r="Y3" s="2" t="n">
-        <v>130</v>
+        <v>120</v>
       </c>
       <c r="Z3" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>slow</t>
         </is>
       </c>
       <c r="AA3" s="2" t="n">
-        <v>0.9</v>
+        <v>0.86</v>
       </c>
       <c r="AB3" s="2" t="n">
-        <v>1.24</v>
+        <v>1.27</v>
       </c>
       <c r="AC3" s="2" t="inlineStr">
         <is>
@@ -1489,34 +1515,38 @@
       <c r="AE3" s="2" t="inlineStr"/>
       <c r="AF3" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>soft</t>
         </is>
       </c>
       <c r="AG3" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="AH3" s="2" t="inlineStr"/>
+        <v>-2</v>
+      </c>
+      <c r="AH3" s="2" t="inlineStr">
+        <is>
+          <t>calme</t>
+        </is>
+      </c>
       <c r="AI3" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ3" s="2" t="n">
-        <v>250</v>
+        <v>700</v>
       </c>
       <c r="AK3" s="2" t="n">
-        <v>280</v>
+        <v>320</v>
       </c>
       <c r="AL3" s="2" t="inlineStr">
         <is>
-          <t>warm</t>
+          <t>focused</t>
         </is>
       </c>
       <c r="AM3" s="2" t="inlineStr">
         <is>
-          <t>rise</t>
+          <t>rising</t>
         </is>
       </c>
       <c r="AN3" s="2" t="n">
-        <v>0.333</v>
+        <v>0.32</v>
       </c>
       <c r="AO3" s="2" t="inlineStr"/>
       <c r="AP3" s="2" t="inlineStr">
@@ -1525,28 +1555,28 @@
         </is>
       </c>
       <c r="AQ3" s="2" t="n">
-        <v>0.9</v>
+        <v>0.86</v>
       </c>
       <c r="AR3" s="2" t="n">
-        <v>0.9</v>
+        <v>0.86</v>
       </c>
       <c r="AS3" s="2" t="n">
-        <v>100</v>
+        <v>82</v>
       </c>
       <c r="AT3" s="2" t="n">
         <v>50</v>
       </c>
       <c r="AU3" s="2" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="AV3" s="2" t="inlineStr">
         <is>
-          <t>question d'écoute, ne change pas le cours</t>
+          <t>arc=indice; intention=faire_deviner; emotion=attention; intensite=1; destinataire=enfant; sous_texte=il_regarde_puis_roule_le_meme_geste; tempo=suspendu; sourire=aucun; respiration=courte_avant_question</t>
         </is>
       </c>
       <c r="AW3" t="inlineStr">
         <is>
-          <t>narrateur|Victorina a besoin de calme.
+          <t>narrateur|Amir a besoin de calme.
 narrateur|Que peut-on faire ?</t>
         </is>
       </c>
@@ -1574,17 +1604,17 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Amir va près d'elle. Il parle tout doux. Une boule. Puis on aplatit. Puis on roule la spirale. Tu as su répéter. Victorina écoute. Elle va observer d'abord. Amir roule une boule douce. Il l'aplatit avec la paume. Il enroule un long boudin. La spirale devient un escargot. Victorina suit des yeux. Observer d'abord, c'est possible. Plus tard, elle pose un doigt. Elle aplatit un tout petit palet. C'est une coquille, ça. Bravo, Amir. Tu as laissé le temps. Le soir, à la maison, papa sort un jeu. Des cartes d'oiseaux sur la nappe. Tu te souviens, Amir ? On pioche. On montre. On pose. C'est répéter, encore. Victorina observe d'abord. Puis elle pioche une carte. C'est un oiseau bleu. Même calme. Autre table.</t>
+          <t>Amir ouvre les mains trop vite. Il veut coller la pâte plate. Les bords se déchirent. Oh. Le sourire ne revient pas. Amir refuse de foncer. Il pose les paumes à plat. Le morceau fendu reste sous ses yeux. Personne ne dit la suite. Il écoute le tic du robinet. Un petit morceau se détache. Les paumes roulent la pâte. Amir s'arrête, il regarde. Une boule. Puis je regarde. Il roule le même geste. La pâte devient ronde, peu à peu. Sur sa boule, l'éclat de boule revient. Elle est ronde, Amir ? Comme la goutte. Merci, Amir. Papa a regardé jusqu'au bout. Amir pose la boule sur la planche. La planche est sous la vitre. On rentre ? La boule vient avec nous. Je la porte, à deux mains. Pas trop vite. Dehors, le chemin sent la terre mouillée. La pluie a laissé des ronds. Des gouttes, papa. Des ronds, comme ta boule. La boule reste ronde, contre la paume. À la maison, la cuisine est tiède. La porte, Amir. Je la pousse. La cuisine sent le bois. Maman pose la boule près de la vitre. Tu veux de l'eau ? Oui, maman. Papa pose un tas de pâte sur la table. Je veux une autre, maintenant ! Le ventre d'Amir se desserre.</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Amir va près d'elle. Il parle tout doux. Une boule. Puis on aplatit. Puis on roule la spirale. Tu as su répéter. Victorina écoute. Elle va observer d'abord. Amir roule une boule douce. Il l'aplatit avec la paume. Il enroule un long boudin. La spirale devient un escargot. Victorina suit des yeux. Observer d'abord, c'est possible. Plus tard, elle pose un doigt. Elle aplatit un tout petit palet. C'est une coquille, ça. Bravo, Amir. Tu as laissé le temps. Le soir, à la maison, papa sort un jeu. Des cartes d'oiseaux sur la nappe. Tu te souviens, Amir ? On pioche. On montre. On pose. C'est répéter, encore. Victorina observe d'abord. Puis elle pioche une carte. C'est un oiseau bleu. Même calme. Autre table.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Amir ouvre les mains trop vite. Il veut coller la pâte plate. Les bords se déchirent. Oh. Le sourire ne revient pas. Amir refuse de foncer. Il pose les paumes à plat. Le morceau fendu reste sous ses yeux. Personne ne dit la suite. Il écoute le tic du robinet. Un petit morceau se détache. Les paumes roulent la pâte. Amir s'arrête, il regarde. Une boule. Puis je regarde. Il roule le &lt;emphasis level="moderate"&gt;même geste&lt;/emphasis&gt;. La pâte devient ronde, peu à peu. Sur sa boule, l'éclat de boule revient. Elle est ronde, Amir ? Comme la goutte. Merci, Amir. Papa a regardé jusqu'au bout. Amir pose la boule sur la planche. La planche est sous la vitre. On rentre ? La boule vient avec nous. Je la porte, à deux mains. Pas trop vite. Dehors, le chemin sent la terre mouillée. La pluie a laissé des ronds. Des gouttes, papa. Des ronds, comme ta boule. La boule reste ronde, contre la paume. À la maison, la cuisine est tiède. La porte, Amir. Je la pousse. La cuisine sent le bois. Maman pose la boule près de la vitre. Tu veux de l'eau ? Oui, maman. Papa pose un tas de pâte sur la table. Je veux une autre, maintenant ! Le ventre d'Amir se desserre.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>Léo a su &lt;emphasis&gt;répéter&lt;/emphasis&gt;. Amina a pu observer d'abord. À l'école, puis à la maison. [pause]</t>
+          <t>Amir ouvre les mains trop vite. Il veut coller la pâte plate. Les bords se déchirent. Oh. Le sourire ne revient pas. Amir refuse de foncer. Il pose les paumes à plat. Le morceau fendu reste sous ses yeux. Personne ne dit la suite. Il écoute le tic du robinet. Un petit morceau se détache. Les paumes roulent la pâte. Amir s'arrête, il regarde. Une boule. Puis je regarde. Il roule le &lt;emphasis&gt;même geste&lt;/emphasis&gt;. La pâte devient ronde, peu à peu. Sur sa boule, l'éclat de boule revient. Elle est ronde, Amir ? Comme la goutte. Merci, Amir. Papa a regardé jusqu'au bout. Amir pose la boule sur la planche. La planche est sous la vitre. On rentre ? La boule vient avec nous. Je la porte, à deux mains. Pas trop vite. Dehors, le chemin sent la terre mouillée. La pluie a laissé des ronds. Des gouttes, papa. Des ronds, comme ta boule. La boule reste ronde, contre la paume. À la maison, la cuisine est tiède. La porte, Amir. Je la pousse. La cuisine sent le bois. Maman pose la boule près de la vitre. Tu veux de l'eau ? Oui, maman. Papa pose un tas de pâte sur la table. Je veux une autre, maintenant ! Le ventre d'Amir se desserre. [pause]</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr"/>
@@ -1631,7 +1661,7 @@
         </is>
       </c>
       <c r="Y4" s="2" t="n">
-        <v>148</v>
+        <v>140</v>
       </c>
       <c r="Z4" s="2" t="inlineStr">
         <is>
@@ -1639,10 +1669,10 @@
         </is>
       </c>
       <c r="AA4" s="2" t="n">
-        <v>0.96</v>
+        <v>0.97</v>
       </c>
       <c r="AB4" s="2" t="n">
-        <v>1.22</v>
+        <v>1.14</v>
       </c>
       <c r="AC4" s="2" t="inlineStr">
         <is>
@@ -1665,30 +1695,30 @@
       </c>
       <c r="AH4" s="2" t="inlineStr">
         <is>
-          <t>répéter</t>
+          <t>même geste</t>
         </is>
       </c>
       <c r="AI4" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ4" s="2" t="n">
-        <v>450</v>
+        <v>560</v>
       </c>
       <c r="AK4" s="2" t="n">
-        <v>280</v>
+        <v>270</v>
       </c>
       <c r="AL4" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>bright</t>
         </is>
       </c>
       <c r="AM4" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN4" s="2" t="n">
-        <v>0.333</v>
+        <v>0.35</v>
       </c>
       <c r="AO4" s="2" t="inlineStr"/>
       <c r="AP4" s="2" t="inlineStr">
@@ -1697,10 +1727,10 @@
         </is>
       </c>
       <c r="AQ4" s="2" t="n">
-        <v>0.96</v>
+        <v>0.97</v>
       </c>
       <c r="AR4" s="2" t="n">
-        <v>0.96</v>
+        <v>0.97</v>
       </c>
       <c r="AS4" s="2" t="n">
         <v>100</v>
@@ -1713,47 +1743,59 @@
       </c>
       <c r="AV4" s="2" t="inlineStr">
         <is>
-          <t>confirmation ; le moteur peut dire engine_ok/near avant ce chunk</t>
+          <t>arc=résolution; intention=faire_vivre_le_geste; emotion=retenue puis fierté_calme; intensite=2; destinataire=enfant; sous_texte=il_regarde_puis_roule_pareil; tempo=naturel; sourire=léger; respiration=relâchée</t>
         </is>
       </c>
       <c r="AW4" t="inlineStr">
         <is>
-          <t>narrateur|Amir va près d'elle.
-narrateur|Il parle tout doux.
+          <t>narrateur|Amir ouvre les mains trop vite.
+narrateur|Il veut coller la pâte plate.
+narrateur|Les bords se déchirent.
+enfant-m|Oh.
+narrateur|Le sourire ne revient pas.
+narrateur|Amir refuse de foncer.
+narrateur|Il pose les paumes à plat.
+narrateur|Le morceau fendu reste sous ses yeux.
+narrateur|Personne ne dit la suite.
+narrateur|Il écoute le tic du robinet.
+narrateur|Un petit morceau se détache.
+narrateur|Les paumes roulent la pâte.
+narrateur|Amir s'arrête, il regarde.
 enfant-m|Une boule.
-enfant-m|Puis on aplatit.
-enfant-m|Puis on roule la spirale.
-maman|Tu as su répéter.
-narrateur|Victorina écoute.
-narrateur|Elle va observer d'abord.
-narrateur|Amir roule une boule douce.
-narrateur|Il l'aplatit avec la paume.
-narrateur|Il enroule un long boudin.
-narrateur|La spirale devient un escargot.
-narrateur|Victorina suit des yeux.
-maman|Observer d'abord, c'est possible.
-narrateur|Plus tard, elle pose un doigt.
-narrateur|Elle aplatit un tout petit palet.
-enfant-m|C'est une coquille, ça.
-maman|Bravo, Amir.
-maman|Tu as laissé le temps.
-narrateur|Le soir, à la maison, papa sort un jeu.
-narrateur|Des cartes d'oiseaux sur la nappe.
-papa|Tu te souviens, Amir ?
-enfant-m|On pioche.
-enfant-m|On montre.
-enfant-m|On pose.
-narrateur|C'est répéter, encore.
-narrateur|Victorina observe d'abord.
-narrateur|Puis elle pioche une carte.
-narrateur|C'est un oiseau bleu.
-papa|Même calme.
-papa|Autre table.</t>
+enfant-m|Puis je regarde.
+narrateur|Il roule le même geste.
+narrateur|La pâte devient ronde, peu à peu.
+narrateur|Sur sa boule, l'éclat de boule revient.
+maman|Elle est ronde, Amir ?
+enfant-m|Comme la goutte.
+papa|Merci, Amir.
+narrateur|Papa a regardé jusqu'au bout.
+narrateur|Amir pose la boule sur la planche.
+narrateur|La planche est sous la vitre.
+maman|On rentre ?
+enfant-m|La boule vient avec nous.
+maman|Je la porte, à deux mains.
+enfant-m|Pas trop vite.
+narrateur|Dehors, le chemin sent la terre mouillée.
+narrateur|La pluie a laissé des ronds.
+enfant-m|Des gouttes, papa.
+papa|Des ronds, comme ta boule.
+narrateur|La boule reste ronde, contre la paume.
+narrateur|À la maison, la cuisine est tiède.
+papa|La porte, Amir.
+papa|Je la pousse.
+enfant-m|La cuisine sent le bois.
+narrateur|Maman pose la boule près de la vitre.
+maman|Tu veux de l'eau ?
+enfant-m|Oui, maman.
+narrateur|Papa pose un tas de pâte sur la table.
+enfant-m|Je veux une autre, maintenant !
+narrateur|Le ventre d'Amir se desserre.</t>
         </is>
       </c>
       <c r="AX4" t="inlineStr">
         <is>
-          <t>pate,cartes</t>
+          <t>pate</t>
         </is>
       </c>
     </row>
@@ -1780,17 +1822,17 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>L'escargot sèche sur une assiette. La spirale tient, tout nette. Tu as fini de ranger les cartes, Amir ? Oui, papa. L'oiseau bleu est reposé. Victorina a regardé d'abord. Oui. À l'atelier, puis ici. La lampe fait un rond jaune. Le rond touche l'assiette. On dirait une coquille, aussi. Comme l'escargot. On a pris le temps. L'arrosoir ne goutte plus. La nappe redevient lisse. La spirale est à moi. Oui. Elle sèche jusqu'à demain.</t>
+          <t>Amir veut la deuxième boule, d'un coup. Il pousse la pâte trop vite. La boule file vers le bord. Ça roule ! Elle s'arrête près de la vitre. Amir veut la rattraper, d'un coup. Amir refuse de foncer. Ses épaules se serrent un peu. Ça tape, dans sa poitrine. Personne ne dit la suite. Il regarde la boule au bord. La cuisine fait tic, un instant. Le robinet de la maison répond. Comme à l'atelier, papa ! Tu l'entends, toi ? Oui, le tic. Amir regarde la première boule. Elle est ronde, près de la vitre. Amir reprend la pâte, plus lentement. Il roule le même geste. Il s'arrête, il regarde. La deuxième boule tient, ronde. Les deux sont près de la vitre ? Oui, maman. Tes pieds sont sous la table ? Oui, papa. Il s'assoit au bord de la chaise. Les deux boules se tiennent. Le tic continue, petit. Le tic est là. Les boules, elles, restent.</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>L'escargot sèche sur une assiette. La spirale tient, tout nette. Tu as fini de ranger les cartes, Amir ? Oui, papa. L'oiseau bleu est reposé. Victorina a regardé d'abord. Oui. À l'atelier, puis ici. La lampe fait un rond jaune. Le rond touche l'assiette. On dirait une coquille, aussi. Comme l'escargot. On a pris le temps. L'arrosoir ne goutte plus. La nappe redevient lisse. La spirale est à moi. Oui. Elle sèche jusqu'à demain.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Amir veut la deuxième &lt;emphasis level="moderate"&gt;boule&lt;/emphasis&gt;, d'un coup. Il pousse la pâte trop vite. La boule file vers le bord. Ça roule ! Elle s'arrête près de la vitre. Amir veut la rattraper, d'un coup. Amir refuse de foncer. Ses épaules se serrent un peu. Ça tape, dans sa poitrine. Personne ne dit la suite. Il regarde la boule au bord. La cuisine fait tic, un instant. Le robinet de la maison répond. Comme à l'atelier, papa ! Tu l'entends, toi ? Oui, le tic. Amir regarde la première boule. Elle est ronde, près de la vitre. Amir reprend la pâte, plus lentement. Il roule le même geste. Il s'arrête, il regarde. La deuxième boule tient, ronde. Les deux sont près de la vitre ? Oui, maman. Tes pieds sont sous la table ? Oui, papa. Il s'assoit au bord de la chaise. Les deux boules se tiennent. Le tic continue, petit. Le tic est là. Les boules, elles, restent.&lt;/prosody&gt;&lt;break time="420ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>Amina pose sa carte. Papa range le jeu. [pause]</t>
+          <t>Amir veut la deuxième &lt;emphasis&gt;boule&lt;/emphasis&gt;, d'un coup. Il pousse la pâte trop vite. La boule file vers le bord. Ça roule ! Elle s'arrête près de la vitre. Amir veut la rattraper, d'un coup. Amir refuse de foncer. Ses épaules se serrent un peu. Ça tape, dans sa poitrine. Personne ne dit la suite. Il regarde la boule au bord. La cuisine fait tic, un instant. Le robinet de la maison répond. Comme à l'atelier, papa ! Tu l'entends, toi ? Oui, le tic. Amir regarde la première boule. Elle est ronde, près de la vitre. Amir reprend la pâte, plus lentement. Il roule le même geste. Il s'arrête, il regarde. La deuxième boule tient, ronde. Les deux sont près de la vitre ? Oui, maman. Tes pieds sont sous la table ? Oui, papa. Il s'assoit au bord de la chaise. Les deux boules se tiennent. Le tic continue, petit. Le tic est là. Les boules, elles, restent. [pause]</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr"/>
@@ -1837,7 +1879,7 @@
         </is>
       </c>
       <c r="Y5" s="2" t="n">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="Z5" s="2" t="inlineStr">
         <is>
@@ -1845,10 +1887,10 @@
         </is>
       </c>
       <c r="AA5" s="2" t="n">
-        <v>0.96</v>
+        <v>1</v>
       </c>
       <c r="AB5" s="2" t="n">
-        <v>1.22</v>
+        <v>1.1</v>
       </c>
       <c r="AC5" s="2" t="inlineStr">
         <is>
@@ -1869,28 +1911,32 @@
       <c r="AG5" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="AH5" s="2" t="inlineStr"/>
+      <c r="AH5" s="2" t="inlineStr">
+        <is>
+          <t>boule</t>
+        </is>
+      </c>
       <c r="AI5" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ5" s="2" t="n">
-        <v>450</v>
+        <v>420</v>
       </c>
       <c r="AK5" s="2" t="n">
-        <v>280</v>
+        <v>250</v>
       </c>
       <c r="AL5" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>lively</t>
         </is>
       </c>
       <c r="AM5" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>dynamic</t>
         </is>
       </c>
       <c r="AN5" s="2" t="n">
-        <v>0.333</v>
+        <v>0.37</v>
       </c>
       <c r="AO5" s="2" t="inlineStr"/>
       <c r="AP5" s="2" t="inlineStr">
@@ -1899,10 +1945,10 @@
         </is>
       </c>
       <c r="AQ5" s="2" t="n">
-        <v>0.96</v>
+        <v>1</v>
       </c>
       <c r="AR5" s="2" t="n">
-        <v>0.96</v>
+        <v>1</v>
       </c>
       <c r="AS5" s="2" t="n">
         <v>100</v>
@@ -1913,32 +1959,49 @@
       <c r="AU5" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="AV5" s="2" t="inlineStr"/>
+      <c r="AV5" s="2" t="inlineStr">
+        <is>
+          <t>arc=action; intention=entraîner; emotion=élan puis prudence; intensite=2; destinataire=enfant; sous_texte=il_refuse_de_rattraper_trop_vite; tempo=vif puis posé; sourire=léger; respiration=courte</t>
+        </is>
+      </c>
       <c r="AW5" t="inlineStr">
         <is>
-          <t>narrateur|L'escargot sèche sur une assiette.
-narrateur|La spirale tient, tout nette.
-papa|Tu as fini de ranger les cartes, Amir ?
+          <t>narrateur|Amir veut la deuxième boule, d'un coup.
+narrateur|Il pousse la pâte trop vite.
+narrateur|La boule file vers le bord.
+enfant-m|Ça roule !
+narrateur|Elle s'arrête près de la vitre.
+narrateur|Amir veut la rattraper, d'un coup.
+narrateur|Amir refuse de foncer.
+narrateur|Ses épaules se serrent un peu.
+narrateur|Ça tape, dans sa poitrine.
+narrateur|Personne ne dit la suite.
+narrateur|Il regarde la boule au bord.
+narrateur|La cuisine fait tic, un instant.
+narrateur|Le robinet de la maison répond.
+enfant-m|Comme à l'atelier, papa !
+papa|Tu l'entends, toi ?
+enfant-m|Oui, le tic.
+narrateur|Amir regarde la première boule.
+narrateur|Elle est ronde, près de la vitre.
+narrateur|Amir reprend la pâte, plus lentement.
+narrateur|Il roule le même geste.
+narrateur|Il s'arrête, il regarde.
+narrateur|La deuxième boule tient, ronde.
+maman|Les deux sont près de la vitre ?
+enfant-m|Oui, maman.
+papa|Tes pieds sont sous la table ?
 enfant-m|Oui, papa.
-maman|L'oiseau bleu est reposé.
-enfant-m|Victorina a regardé d'abord.
-papa|Oui.
-papa|À l'atelier, puis ici.
-narrateur|La lampe fait un rond jaune.
-narrateur|Le rond touche l'assiette.
-maman|On dirait une coquille, aussi.
-enfant-m|Comme l'escargot.
-papa|On a pris le temps.
-narrateur|L'arrosoir ne goutte plus.
-narrateur|La nappe redevient lisse.
-enfant-m|La spirale est à moi.
-maman|Oui.
-maman|Elle sèche jusqu'à demain.</t>
+narrateur|Il s'assoit au bord de la chaise.
+narrateur|Les deux boules se tiennent.
+narrateur|Le tic continue, petit.
+papa|Le tic est là.
+enfant-m|Les boules, elles, restent.</t>
         </is>
       </c>
       <c r="AX5" t="inlineStr">
         <is>
-          <t>assiette,cartes</t>
+          <t>pate,table</t>
         </is>
       </c>
     </row>
@@ -1965,17 +2028,17 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>L'escargot repose sur l'assiette. La spirale est sèche, presque. Bonne soirée, Amir. L'oiseau bleu est rangé.</t>
+          <t>Ils restent près de la table. Les deux boules reposent près de la vitre. L'éclat est là, papa. Tu le vois sur la pâte ? Oui, papa. On est bien, ici. La vitre fait un rond, plus petit. La cuisine sent la terre, un peu. Elle est ronde, ma boule. Elle est ronde, Amir. Oui, maman. Amir pose la joue près de la pâte. La pâte est froide, un peu. C'est froid. Tu le sens sur tes joues ? Oui, elle est froide. La première boule porte une trace de paume. Dehors, la cour s'endort. L'éclat de boule tient sur la pâte.</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>L'escargot repose sur l'assiette. La spirale est sèche, presque. Bonne soirée, Amir. L'oiseau bleu est rangé.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Ils restent près de la table. Les deux boules reposent près de la vitre. L'éclat est là, papa. Tu le vois sur la pâte ? Oui, papa. On est bien, ici. La vitre fait un rond, plus petit. La cuisine sent la terre, un peu. Elle est ronde, ma boule. Elle est ronde, Amir. Oui, maman. Amir pose la joue près de la pâte. La pâte est froide, un peu. C'est froid. Tu le sens sur tes joues ? Oui, elle est froide. La première boule porte une trace de paume. Dehors, la cour s'endort. L'&lt;emphasis level="moderate"&gt;éclat de boule&lt;/emphasis&gt; tient sur la pâte.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>&lt;lower-pitch&gt;&lt;soft&gt;L'histoire est finie.&lt;/soft&gt;&lt;/lower-pitch&gt; [pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Ils restent près de la table. Les deux boules reposent près de la vitre. L'éclat est là, papa. Tu le vois sur la pâte ? Oui, papa. On est bien, ici. La vitre fait un rond, plus petit. La cuisine sent la terre, un peu. Elle est ronde, ma boule. Elle est ronde, Amir. Oui, maman. Amir pose la joue près de la pâte. La pâte est froide, un peu. C'est froid. Tu le sens sur tes joues ? Oui, elle est froide. La première boule porte une trace de paume. Dehors, la cour s'endort. L'&lt;emphasis&gt;éclat de boule&lt;/emphasis&gt; tient sur la pâte.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr"/>
@@ -2022,18 +2085,18 @@
         </is>
       </c>
       <c r="Y6" s="2" t="n">
-        <v>136</v>
+        <v>118</v>
       </c>
       <c r="Z6" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>slow</t>
         </is>
       </c>
       <c r="AA6" s="2" t="n">
-        <v>0.92</v>
+        <v>0.85</v>
       </c>
       <c r="AB6" s="2" t="n">
-        <v>1.2</v>
+        <v>1.28</v>
       </c>
       <c r="AC6" s="2" t="inlineStr">
         <is>
@@ -2042,12 +2105,12 @@
       </c>
       <c r="AD6" s="2" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>-2st</t>
         </is>
       </c>
       <c r="AE6" s="2" t="inlineStr">
         <is>
-          <t>lower-pitch</t>
+          <t>low-pitch</t>
         </is>
       </c>
       <c r="AF6" s="2" t="inlineStr">
@@ -2056,17 +2119,21 @@
         </is>
       </c>
       <c r="AG6" s="2" t="n">
-        <v>-2</v>
-      </c>
-      <c r="AH6" s="2" t="inlineStr"/>
+        <v>-3</v>
+      </c>
+      <c r="AH6" s="2" t="inlineStr">
+        <is>
+          <t>éclat de boule</t>
+        </is>
+      </c>
       <c r="AI6" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ6" s="2" t="n">
-        <v>600</v>
+        <v>900</v>
       </c>
       <c r="AK6" s="2" t="n">
-        <v>280</v>
+        <v>340</v>
       </c>
       <c r="AL6" s="2" t="inlineStr">
         <is>
@@ -2075,11 +2142,11 @@
       </c>
       <c r="AM6" s="2" t="inlineStr">
         <is>
-          <t>fall</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN6" s="2" t="n">
-        <v>0.333</v>
+        <v>0.31</v>
       </c>
       <c r="AO6" s="2" t="inlineStr"/>
       <c r="AP6" s="2" t="inlineStr">
@@ -2088,27 +2155,46 @@
         </is>
       </c>
       <c r="AQ6" s="2" t="n">
-        <v>0.92</v>
+        <v>0.85</v>
       </c>
       <c r="AR6" s="2" t="n">
-        <v>0.92</v>
+        <v>0.85</v>
       </c>
       <c r="AS6" s="2" t="n">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="AT6" s="2" t="n">
-        <v>35</v>
+        <v>42</v>
       </c>
       <c r="AU6" s="2" t="n">
-        <v>8</v>
-      </c>
-      <c r="AV6" s="2" t="inlineStr"/>
+        <v>12</v>
+      </c>
+      <c r="AV6" s="2" t="inlineStr">
+        <is>
+          <t>arc=retour; intention=refermer; emotion=tendresse et fierté_calme; intensite=1; destinataire=enfant; sous_texte=l_eclat_du_debut_tient_sur_la_pate; tempo=posé; sourire=léger; respiration=ample</t>
+        </is>
+      </c>
       <c r="AW6" t="inlineStr">
         <is>
-          <t>narrateur|L'escargot repose sur l'assiette.
-narrateur|La spirale est sèche, presque.
-maman|Bonne soirée, Amir.
-papa|L'oiseau bleu est rangé.</t>
+          <t>narrateur|Ils restent près de la table.
+narrateur|Les deux boules reposent près de la vitre.
+enfant-m|L'éclat est là, papa.
+papa|Tu le vois sur la pâte ?
+enfant-m|Oui, papa.
+maman|On est bien, ici.
+narrateur|La vitre fait un rond, plus petit.
+narrateur|La cuisine sent la terre, un peu.
+enfant-m|Elle est ronde, ma boule.
+maman|Elle est ronde, Amir.
+enfant-m|Oui, maman.
+narrateur|Amir pose la joue près de la pâte.
+narrateur|La pâte est froide, un peu.
+enfant-m|C'est froid.
+papa|Tu le sens sur tes joues ?
+enfant-m|Oui, elle est froide.
+narrateur|La première boule porte une trace de paume.
+narrateur|Dehors, la cour s'endort.
+narrateur|L'éclat de boule tient sur la pâte.</t>
         </is>
       </c>
     </row>
@@ -2129,7 +2215,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A12"/>
+  <dimension ref="A1:A13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -2214,6 +2300,13 @@
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
+        <is>
+          <t>F-NAR-008 récit, pas une leçon en puces</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
         <is>
           <t>F-NAR-008 récit, pas une leçon en puces</t>
         </is>

</xml_diff>